<commit_message>
Preserve full WBS codes in Gantt display
</commit_message>
<xml_diff>
--- a/08-Project-Schedule/Week08-Project-Schedule-David-Zupinski.xlsx
+++ b/08-Project-Schedule/Week08-Project-Schedule-David-Zupinski.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R8d97a3a2e3bd473e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Schedule" sheetId="2" r:id="Rda80362408de405f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A-D Practice Bridge" sheetId="3" r:id="R72c7338b5789422b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gantt View" sheetId="4" r:id="R25f35f700e494b45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="Rc23404ac2c83464f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Schedule" sheetId="2" r:id="R14b78c85a9494cfa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A-D Practice Bridge" sheetId="3" r:id="Ra5295c97e00f4901"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gantt View" sheetId="4" r:id="R1a0f76e87c254524"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -215,13 +215,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="6">
+  <x:numFmts count="7">
     <x:numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <x:numFmt numFmtId="41" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
     <x:numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <x:numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <x:numFmt numFmtId="200" formatCode="@"/>
-    <x:numFmt numFmtId="201" formatCode="0;-0;;@"/>
+    <x:numFmt numFmtId="201" formatCode="0.0#########;-0.0#########;;@"/>
+    <x:numFmt numFmtId="202" formatCode="0;-0;;@"/>
   </x:numFmts>
   <x:fonts count="30">
     <x:font>
@@ -538,7 +539,7 @@
     <x:xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <x:xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="95">
+  <x:cellXfs count="97">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
@@ -810,6 +811,10 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="6">
     <x:cellStyle name="Comma" xfId="1"/>
@@ -2960,15 +2965,15 @@
         <x:f>'Project Schedule'!A3</x:f>
         <x:v>1.0</x:v>
       </x:c>
-      <x:c r="B5" s="93" t="str">
+      <x:c r="B5" s="95" t="str">
         <x:f>'Project Schedule'!B3</x:f>
         <x:v>PLANNING AND SCOPE BASELINE</x:v>
       </x:c>
-      <x:c r="C5" s="93" t="str">
+      <x:c r="C5" s="95" t="str">
         <x:f>'Project Schedule'!D3</x:f>
         <x:v>Phase Header</x:v>
       </x:c>
-      <x:c r="D5" s="93" t="n">
+      <x:c r="D5" s="95" t="n">
         <x:f>'Project Schedule'!J3</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -3098,15 +3103,15 @@
         <x:f>'Project Schedule'!A4</x:f>
         <x:v>1.1</x:v>
       </x:c>
-      <x:c r="B6" s="93" t="str">
+      <x:c r="B6" s="95" t="str">
         <x:f>'Project Schedule'!B4</x:f>
         <x:v>Confirm shared intake, identity and access rules</x:v>
       </x:c>
-      <x:c r="C6" s="93" t="str">
+      <x:c r="C6" s="95" t="str">
         <x:f>'Project Schedule'!D4</x:f>
         <x:v>Task</x:v>
       </x:c>
-      <x:c r="D6" s="93" t="str">
+      <x:c r="D6" s="95" t="str">
         <x:f>'Project Schedule'!J4</x:f>
         <x:v>YES</x:v>
       </x:c>
@@ -3237,15 +3242,15 @@
         <x:f>'Project Schedule'!A5</x:f>
         <x:v>1.2</x:v>
       </x:c>
-      <x:c r="B7" s="93" t="str">
+      <x:c r="B7" s="95" t="str">
         <x:f>'Project Schedule'!B5</x:f>
         <x:v>Document constraints and acceptance plan</x:v>
       </x:c>
-      <x:c r="C7" s="93" t="str">
+      <x:c r="C7" s="95" t="str">
         <x:f>'Project Schedule'!D5</x:f>
         <x:v>Task</x:v>
       </x:c>
-      <x:c r="D7" s="93" t="str">
+      <x:c r="D7" s="95" t="str">
         <x:f>'Project Schedule'!J5</x:f>
         <x:v>YES</x:v>
       </x:c>
@@ -3376,15 +3381,15 @@
         <x:f>'Project Schedule'!A6</x:f>
         <x:v>1.3</x:v>
       </x:c>
-      <x:c r="B8" s="93" t="str">
+      <x:c r="B8" s="95" t="str">
         <x:f>'Project Schedule'!B6</x:f>
         <x:v>Scope and delivery baseline approved</x:v>
       </x:c>
-      <x:c r="C8" s="93" t="str">
+      <x:c r="C8" s="95" t="str">
         <x:f>'Project Schedule'!D6</x:f>
         <x:v>Milestone</x:v>
       </x:c>
-      <x:c r="D8" s="93" t="n">
+      <x:c r="D8" s="95" t="n">
         <x:f>'Project Schedule'!J6</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -3515,15 +3520,15 @@
         <x:f>'Project Schedule'!A7</x:f>
         <x:v>2.0</x:v>
       </x:c>
-      <x:c r="B9" s="93" t="str">
+      <x:c r="B9" s="95" t="str">
         <x:f>'Project Schedule'!B7</x:f>
         <x:v>INTAKE AND SCHEDULING SOLUTION</x:v>
       </x:c>
-      <x:c r="C9" s="93" t="str">
+      <x:c r="C9" s="95" t="str">
         <x:f>'Project Schedule'!D7</x:f>
         <x:v>Phase Header</x:v>
       </x:c>
-      <x:c r="D9" s="93" t="n">
+      <x:c r="D9" s="95" t="n">
         <x:f>'Project Schedule'!J7</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -3653,15 +3658,15 @@
         <x:f>'Project Schedule'!A8</x:f>
         <x:v>2.1</x:v>
       </x:c>
-      <x:c r="B10" s="93" t="str">
+      <x:c r="B10" s="95" t="str">
         <x:f>'Project Schedule'!B8</x:f>
         <x:v>Configure intake and retained-data workflow</x:v>
       </x:c>
-      <x:c r="C10" s="93" t="str">
+      <x:c r="C10" s="95" t="str">
         <x:f>'Project Schedule'!D8</x:f>
         <x:v>Task</x:v>
       </x:c>
-      <x:c r="D10" s="93" t="str">
+      <x:c r="D10" s="95" t="str">
         <x:f>'Project Schedule'!J8</x:f>
         <x:v>YES</x:v>
       </x:c>
@@ -3793,15 +3798,15 @@
         <x:f>'Project Schedule'!A9</x:f>
         <x:v>2.2</x:v>
       </x:c>
-      <x:c r="B11" s="93" t="str">
+      <x:c r="B11" s="95" t="str">
         <x:f>'Project Schedule'!B9</x:f>
         <x:v>Configure clinic/date availability</x:v>
       </x:c>
-      <x:c r="C11" s="93" t="str">
+      <x:c r="C11" s="95" t="str">
         <x:f>'Project Schedule'!D9</x:f>
         <x:v>Task</x:v>
       </x:c>
-      <x:c r="D11" s="93" t="n">
+      <x:c r="D11" s="95" t="n">
         <x:f>'Project Schedule'!J9</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -3932,15 +3937,15 @@
         <x:f>'Project Schedule'!A10</x:f>
         <x:v>2.3.1</x:v>
       </x:c>
-      <x:c r="B12" s="93" t="str">
+      <x:c r="B12" s="95" t="str">
         <x:f>'Project Schedule'!B10</x:f>
         <x:v>Integrate booking and test conflict handling</x:v>
       </x:c>
-      <x:c r="C12" s="93" t="str">
+      <x:c r="C12" s="95" t="str">
         <x:f>'Project Schedule'!D10</x:f>
         <x:v>Task</x:v>
       </x:c>
-      <x:c r="D12" s="93" t="str">
+      <x:c r="D12" s="95" t="str">
         <x:f>'Project Schedule'!J10</x:f>
         <x:v>YES</x:v>
       </x:c>
@@ -4072,15 +4077,15 @@
         <x:f>'Project Schedule'!A11</x:f>
         <x:v>2.3.2</x:v>
       </x:c>
-      <x:c r="B13" s="93" t="str">
+      <x:c r="B13" s="95" t="str">
         <x:f>'Project Schedule'!B11</x:f>
         <x:v>Run cross-clinic acceptance tests</x:v>
       </x:c>
-      <x:c r="C13" s="93" t="str">
+      <x:c r="C13" s="95" t="str">
         <x:f>'Project Schedule'!D11</x:f>
         <x:v>Task</x:v>
       </x:c>
-      <x:c r="D13" s="93" t="str">
+      <x:c r="D13" s="95" t="str">
         <x:f>'Project Schedule'!J11</x:f>
         <x:v>YES</x:v>
       </x:c>
@@ -4211,15 +4216,15 @@
         <x:f>'Project Schedule'!A12</x:f>
         <x:v>2.3.3</x:v>
       </x:c>
-      <x:c r="B14" s="93" t="str">
+      <x:c r="B14" s="95" t="str">
         <x:f>'Project Schedule'!B12</x:f>
         <x:v>Core solution accepted for pilot</x:v>
       </x:c>
-      <x:c r="C14" s="93" t="str">
+      <x:c r="C14" s="95" t="str">
         <x:f>'Project Schedule'!D12</x:f>
         <x:v>Milestone</x:v>
       </x:c>
-      <x:c r="D14" s="93" t="n">
+      <x:c r="D14" s="95" t="n">
         <x:f>'Project Schedule'!J12</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -4350,15 +4355,15 @@
         <x:f>'Project Schedule'!A13</x:f>
         <x:v>3.0</x:v>
       </x:c>
-      <x:c r="B15" s="93" t="str">
+      <x:c r="B15" s="95" t="str">
         <x:f>'Project Schedule'!B13</x:f>
         <x:v>CLINIC READINESS AND ROLLOUT</x:v>
       </x:c>
-      <x:c r="C15" s="93" t="str">
+      <x:c r="C15" s="95" t="str">
         <x:f>'Project Schedule'!D13</x:f>
         <x:v>Phase Header</x:v>
       </x:c>
-      <x:c r="D15" s="93" t="n">
+      <x:c r="D15" s="95" t="n">
         <x:f>'Project Schedule'!J13</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -4488,15 +4493,15 @@
         <x:f>'Project Schedule'!A14</x:f>
         <x:v>3.1.1</x:v>
       </x:c>
-      <x:c r="B16" s="93" t="str">
+      <x:c r="B16" s="95" t="str">
         <x:f>'Project Schedule'!B14</x:f>
         <x:v>Prepare role-based training materials</x:v>
       </x:c>
-      <x:c r="C16" s="93" t="str">
+      <x:c r="C16" s="95" t="str">
         <x:f>'Project Schedule'!D14</x:f>
         <x:v>Task</x:v>
       </x:c>
-      <x:c r="D16" s="93" t="n">
+      <x:c r="D16" s="95" t="n">
         <x:f>'Project Schedule'!J14</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -4628,15 +4633,15 @@
         <x:f>'Project Schedule'!A15</x:f>
         <x:v>3.1.2</x:v>
       </x:c>
-      <x:c r="B17" s="93" t="str">
+      <x:c r="B17" s="95" t="str">
         <x:f>'Project Schedule'!B15</x:f>
         <x:v>Train designated pilot-clinic staff</x:v>
       </x:c>
-      <x:c r="C17" s="93" t="str">
+      <x:c r="C17" s="95" t="str">
         <x:f>'Project Schedule'!D15</x:f>
         <x:v>Task</x:v>
       </x:c>
-      <x:c r="D17" s="93" t="str">
+      <x:c r="D17" s="95" t="str">
         <x:f>'Project Schedule'!J15</x:f>
         <x:v>YES</x:v>
       </x:c>
@@ -4767,15 +4772,15 @@
         <x:f>'Project Schedule'!A16</x:f>
         <x:v>3.2.1</x:v>
       </x:c>
-      <x:c r="B18" s="93" t="str">
+      <x:c r="B18" s="95" t="str">
         <x:f>'Project Schedule'!B16</x:f>
         <x:v>Pilot clinic launched</x:v>
       </x:c>
-      <x:c r="C18" s="93" t="str">
+      <x:c r="C18" s="95" t="str">
         <x:f>'Project Schedule'!D16</x:f>
         <x:v>Milestone</x:v>
       </x:c>
-      <x:c r="D18" s="93" t="n">
+      <x:c r="D18" s="95" t="n">
         <x:f>'Project Schedule'!J16</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -4906,15 +4911,15 @@
         <x:f>'Project Schedule'!A17</x:f>
         <x:v>3.2.2</x:v>
       </x:c>
-      <x:c r="B19" s="93" t="str">
+      <x:c r="B19" s="95" t="str">
         <x:f>'Project Schedule'!B17</x:f>
         <x:v>Observe pilot and resolve rollout blockers</x:v>
       </x:c>
-      <x:c r="C19" s="93" t="str">
+      <x:c r="C19" s="95" t="str">
         <x:f>'Project Schedule'!D17</x:f>
         <x:v>Task</x:v>
       </x:c>
-      <x:c r="D19" s="93" t="str">
+      <x:c r="D19" s="95" t="str">
         <x:f>'Project Schedule'!J17</x:f>
         <x:v>YES</x:v>
       </x:c>
@@ -5049,15 +5054,15 @@
         <x:f>'Project Schedule'!A18</x:f>
         <x:v>3.1.3</x:v>
       </x:c>
-      <x:c r="B20" s="93" t="str">
+      <x:c r="B20" s="95" t="str">
         <x:f>'Project Schedule'!B18</x:f>
         <x:v>Train staff at remaining five clinics</x:v>
       </x:c>
-      <x:c r="C20" s="93" t="str">
+      <x:c r="C20" s="95" t="str">
         <x:f>'Project Schedule'!D18</x:f>
         <x:v>Task</x:v>
       </x:c>
-      <x:c r="D20" s="93" t="n">
+      <x:c r="D20" s="95" t="n">
         <x:f>'Project Schedule'!J18</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -5190,15 +5195,15 @@
         <x:f>'Project Schedule'!A19</x:f>
         <x:v>3.3.1</x:v>
       </x:c>
-      <x:c r="B21" s="93" t="str">
+      <x:c r="B21" s="95" t="str">
         <x:f>'Project Schedule'!B19</x:f>
         <x:v>Deploy and verify remaining five clinics</x:v>
       </x:c>
-      <x:c r="C21" s="93" t="str">
+      <x:c r="C21" s="95" t="str">
         <x:f>'Project Schedule'!D19</x:f>
         <x:v>Task</x:v>
       </x:c>
-      <x:c r="D21" s="93" t="str">
+      <x:c r="D21" s="95" t="str">
         <x:f>'Project Schedule'!J19</x:f>
         <x:v>YES</x:v>
       </x:c>
@@ -5329,15 +5334,15 @@
         <x:f>'Project Schedule'!A20</x:f>
         <x:v>3.3.2</x:v>
       </x:c>
-      <x:c r="B22" s="93" t="str">
+      <x:c r="B22" s="95" t="str">
         <x:f>'Project Schedule'!B20</x:f>
         <x:v>All six clinics live and verified</x:v>
       </x:c>
-      <x:c r="C22" s="93" t="str">
+      <x:c r="C22" s="95" t="str">
         <x:f>'Project Schedule'!D20</x:f>
         <x:v>Milestone</x:v>
       </x:c>
-      <x:c r="D22" s="93" t="n">
+      <x:c r="D22" s="95" t="n">
         <x:f>'Project Schedule'!J20</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -5468,15 +5473,15 @@
         <x:f>'Project Schedule'!A21</x:f>
         <x:v>4.0</x:v>
       </x:c>
-      <x:c r="B23" s="93" t="str">
+      <x:c r="B23" s="95" t="str">
         <x:f>'Project Schedule'!B21</x:f>
         <x:v>POST-LAUNCH SUPPORT AND HANDOFF</x:v>
       </x:c>
-      <x:c r="C23" s="93" t="str">
+      <x:c r="C23" s="95" t="str">
         <x:f>'Project Schedule'!D21</x:f>
         <x:v>Phase Header</x:v>
       </x:c>
-      <x:c r="D23" s="93" t="n">
+      <x:c r="D23" s="95" t="n">
         <x:f>'Project Schedule'!J21</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -5606,15 +5611,15 @@
         <x:f>'Project Schedule'!A22</x:f>
         <x:v>4.1</x:v>
       </x:c>
-      <x:c r="B24" s="93" t="str">
+      <x:c r="B24" s="95" t="str">
         <x:f>'Project Schedule'!B22</x:f>
         <x:v>Provide 90-day rollout support</x:v>
       </x:c>
-      <x:c r="C24" s="93" t="str">
+      <x:c r="C24" s="95" t="str">
         <x:f>'Project Schedule'!D22</x:f>
         <x:v>Task</x:v>
       </x:c>
-      <x:c r="D24" s="93" t="str">
+      <x:c r="D24" s="95" t="str">
         <x:f>'Project Schedule'!J22</x:f>
         <x:v>YES</x:v>
       </x:c>
@@ -5757,15 +5762,15 @@
         <x:f>'Project Schedule'!A23</x:f>
         <x:v>4.2</x:v>
       </x:c>
-      <x:c r="B25" s="93" t="str">
+      <x:c r="B25" s="95" t="str">
         <x:f>'Project Schedule'!B23</x:f>
         <x:v>Prepare operating guides and ownership transfer</x:v>
       </x:c>
-      <x:c r="C25" s="93" t="str">
+      <x:c r="C25" s="95" t="str">
         <x:f>'Project Schedule'!D23</x:f>
         <x:v>Task</x:v>
       </x:c>
-      <x:c r="D25" s="93" t="n">
+      <x:c r="D25" s="95" t="n">
         <x:f>'Project Schedule'!J23</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -5897,15 +5902,15 @@
         <x:f>'Project Schedule'!A24</x:f>
         <x:v>4.3.1</x:v>
       </x:c>
-      <x:c r="B26" s="93" t="str">
+      <x:c r="B26" s="95" t="str">
         <x:f>'Project Schedule'!B24</x:f>
         <x:v>Document lessons learned and closure evidence</x:v>
       </x:c>
-      <x:c r="C26" s="93" t="str">
+      <x:c r="C26" s="95" t="str">
         <x:f>'Project Schedule'!D24</x:f>
         <x:v>Task</x:v>
       </x:c>
-      <x:c r="D26" s="93" t="n">
+      <x:c r="D26" s="95" t="n">
         <x:f>'Project Schedule'!J24</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -6037,15 +6042,15 @@
         <x:f>'Project Schedule'!A25</x:f>
         <x:v>4.3.2</x:v>
       </x:c>
-      <x:c r="B27" s="93" t="str">
+      <x:c r="B27" s="95" t="str">
         <x:f>'Project Schedule'!B25</x:f>
         <x:v>Final handoff and closure accepted</x:v>
       </x:c>
-      <x:c r="C27" s="93" t="str">
+      <x:c r="C27" s="95" t="str">
         <x:f>'Project Schedule'!D25</x:f>
         <x:v>Milestone</x:v>
       </x:c>
-      <x:c r="D27" s="93" t="n">
+      <x:c r="D27" s="95" t="n">
         <x:f>'Project Schedule'!J25</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -6176,15 +6181,15 @@
         <x:f>'Project Schedule'!A26</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="B28" s="93" t="n">
+      <x:c r="B28" s="95" t="n">
         <x:f>'Project Schedule'!B26</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C28" s="93" t="n">
+      <x:c r="C28" s="95" t="n">
         <x:f>'Project Schedule'!D26</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D28" s="93" t="n">
+      <x:c r="D28" s="95" t="n">
         <x:f>'Project Schedule'!J26</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -6314,15 +6319,15 @@
         <x:f>'Project Schedule'!A27</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="B29" s="93" t="n">
+      <x:c r="B29" s="95" t="n">
         <x:f>'Project Schedule'!B27</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C29" s="93" t="n">
+      <x:c r="C29" s="95" t="n">
         <x:f>'Project Schedule'!D27</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D29" s="93" t="n">
+      <x:c r="D29" s="95" t="n">
         <x:f>'Project Schedule'!J27</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -6449,33 +6454,33 @@
     </x:row>
     <x:row r="30" ht="32" customHeight="1">
       <x:c r="A30" s="94"/>
-      <x:c r="B30" s="93"/>
-      <x:c r="C30" s="94"/>
-      <x:c r="D30" s="94"/>
+      <x:c r="B30" s="95"/>
+      <x:c r="C30" s="96"/>
+      <x:c r="D30" s="96"/>
     </x:row>
     <x:row r="31" ht="32" customHeight="1">
       <x:c r="A31" s="94"/>
-      <x:c r="B31" s="93"/>
-      <x:c r="C31" s="94"/>
-      <x:c r="D31" s="94"/>
+      <x:c r="B31" s="95"/>
+      <x:c r="C31" s="96"/>
+      <x:c r="D31" s="96"/>
     </x:row>
     <x:row r="32" ht="32" customHeight="1">
       <x:c r="A32" s="94"/>
-      <x:c r="B32" s="93"/>
-      <x:c r="C32" s="94"/>
-      <x:c r="D32" s="94"/>
+      <x:c r="B32" s="95"/>
+      <x:c r="C32" s="96"/>
+      <x:c r="D32" s="96"/>
     </x:row>
     <x:row r="33" ht="32" customHeight="1">
       <x:c r="A33" s="94"/>
-      <x:c r="B33" s="93"/>
-      <x:c r="C33" s="94"/>
-      <x:c r="D33" s="94"/>
+      <x:c r="B33" s="95"/>
+      <x:c r="C33" s="96"/>
+      <x:c r="D33" s="96"/>
     </x:row>
     <x:row r="34" ht="32" customHeight="1">
       <x:c r="A34" s="94"/>
-      <x:c r="B34" s="93"/>
-      <x:c r="C34" s="94"/>
-      <x:c r="D34" s="94"/>
+      <x:c r="B34" s="95"/>
+      <x:c r="C34" s="96"/>
+      <x:c r="D34" s="96"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>